<commit_message>
Corrige conflito de rota: move financeiro e gabinete para (dashboard)
Páginas criadas em /financeiro e /gabinete conflitavam com as existentes
em /(dashboard)/financeiro e /(dashboard)/gabinete no Next.js App Router.
Move o conteúdo novo para o local correto e remove os duplicados.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prospeccao_Eleitoral_2026_JF.xlsx
+++ b/Prospeccao_Eleitoral_2026_JF.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -143,6 +143,12 @@
       <color rgb="FF222222"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -202,7 +208,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -238,11 +244,55 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -383,6 +433,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -854,6 +912,8 @@
           <t>ATENCAO: Telefone, WhatsApp, Endereco, Presidente e Assessor devem ser preenchidos manualmente apos pesquisa presencial ou via SGIP do TSE.</t>
         </is>
       </c>
+      <c r="C12" s="48" t="n"/>
+      <c r="D12" s="49" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="9" t="inlineStr">
@@ -861,6 +921,8 @@
           <t>Fonte oficial SGIP: https://sgip3.tse.jus.br/sgip3-consulta  |  TRE-MG: https://www.tre-mg.jus.br/partidos/partidos-politicos</t>
         </is>
       </c>
+      <c r="C13" s="48" t="n"/>
+      <c r="D13" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1269,6 +1331,11 @@
           <t>STATUS:  Concluido  |  Em andamento  |  Pendente  |  Bloqueado</t>
         </is>
       </c>
+      <c r="C15" s="48" t="n"/>
+      <c r="D15" s="48" t="n"/>
+      <c r="E15" s="48" t="n"/>
+      <c r="F15" s="48" t="n"/>
+      <c r="G15" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1324,6 +1391,18 @@
           <t>ATENCAO: Telefone, WhatsApp, Endereco, Presidente e Assessor mudam frequentemente. Confirme via SGIP (sgip3.tse.jus.br) ou pesquisa presencial.</t>
         </is>
       </c>
+      <c r="B3" s="48" t="n"/>
+      <c r="C3" s="48" t="n"/>
+      <c r="D3" s="48" t="n"/>
+      <c r="E3" s="48" t="n"/>
+      <c r="F3" s="48" t="n"/>
+      <c r="G3" s="48" t="n"/>
+      <c r="H3" s="48" t="n"/>
+      <c r="I3" s="48" t="n"/>
+      <c r="J3" s="48" t="n"/>
+      <c r="K3" s="48" t="n"/>
+      <c r="L3" s="48" t="n"/>
+      <c r="M3" s="49" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
@@ -1411,34 +1490,34 @@
           <t>Centro-Esquerda</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F5" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G5" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>juizdefora.mg.pt.org.br</t>
-        </is>
-      </c>
-      <c r="I5" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J5" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Av. Olegário Maciel, 1159 - Centro  CEP 36016-010</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99986-4698</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99986-4698</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>dmptjf@gmail.com</t>
+        </is>
+      </c>
+      <c r="I5" s="30" t="inlineStr">
+        <is>
+          <t>Fabiana Rabelo dos Santos Nascimento</t>
+        </is>
+      </c>
+      <c r="J5" s="30" t="inlineStr">
+        <is>
+          <t>Daniela de Oliveira Paiva (Sec. Organização)</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
@@ -1474,34 +1553,34 @@
           <t>Direita</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F6" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
-        <is>
-          <t>pl.org.br</t>
-        </is>
-      </c>
-      <c r="I6" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J6" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Rua Floriano Peixoto, 536 - Loja 1 - Centro  CEP 36015-440</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98874-7308</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98874-7308</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>charllesevangelista@yahoo.com.br</t>
+        </is>
+      </c>
+      <c r="I6" s="30" t="inlineStr">
+        <is>
+          <t>Charlles Thomacelli Evangelista</t>
+        </is>
+      </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K6" s="28" t="inlineStr">
@@ -1537,34 +1616,34 @@
           <t>Centro-Esquerda</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F7" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G7" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>psb.org.br</t>
-        </is>
-      </c>
-      <c r="I7" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J7" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Rua Mariano Fontes, 15 - Cerâmica  CEP 36080-390</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99156-3473</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99156-3473</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>paulaassuimpcao@yahoo.com.br</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>Paula Michelle de Oliveira Assumpção</t>
+        </is>
+      </c>
+      <c r="J7" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -1600,34 +1679,34 @@
           <t>Centro</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G8" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H8" s="24" t="inlineStr">
-        <is>
-          <t>mdb.org.br</t>
-        </is>
-      </c>
-      <c r="I8" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J8" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Praça da República, 217 - Poço Rico  CEP 36020-060</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99988-2095</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99988-2095</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>joaocesarnovais@gmail.com</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="inlineStr">
+        <is>
+          <t>João Cesar de Novais</t>
+        </is>
+      </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>Luiz Carlos Carvalho (Tesoureiro)</t>
         </is>
       </c>
       <c r="K8" s="28" t="inlineStr">
@@ -1726,34 +1805,34 @@
           <t>Centro-Direita</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>uniaobrasil.org.br</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J10" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Rua Benjamin Constant, 983 - Apto 203 - Santa Cecília  CEP 36015-400</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99987-7060</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99987-7060</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>antonioaguiar54@gmail.com</t>
+        </is>
+      </c>
+      <c r="I10" s="30" t="inlineStr">
+        <is>
+          <t>Antonio Santos de Aguiar</t>
+        </is>
+      </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K10" s="28" t="inlineStr">
@@ -1789,34 +1868,34 @@
           <t>Centro-Direita</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>psd-mg.org.br</t>
-        </is>
-      </c>
-      <c r="I11" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J11" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Rua Alexandre Vicentin, 135 - São Bernardo  CEP 36090-400</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>(32) 98854-4480</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>(32) 98854-4480</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>atila.presidente.psd@gmail.com</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>Átila Henrique de Faria</t>
+        </is>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K11" s="25" t="inlineStr">
@@ -1978,34 +2057,34 @@
           <t>Centro-Esquerda</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F14" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G14" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H14" s="24" t="inlineStr">
-        <is>
-          <t>pv.org.br</t>
-        </is>
-      </c>
-      <c r="I14" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J14" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Av. Pedro Afonso Pinheiro, 257 - Santa Efigênia  CEP 36032-280</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98813-1365</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98813-1365</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>negrobussola29@gmail.com</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>Jefferson da Silva Januário</t>
+        </is>
+      </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t>Francisco Marcos Fonseca de Assis (Sec. Finanças)</t>
         </is>
       </c>
       <c r="K14" s="28" t="inlineStr">
@@ -2104,34 +2183,34 @@
           <t>Esquerda</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H16" s="24" t="inlineStr">
-        <is>
-          <t>pcdob.org.br</t>
-        </is>
-      </c>
-      <c r="I16" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J16" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Rua Prof. José Barata, 816 - Santos Dumont  CEP 36038-100</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99103-4805</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>(32) 99103-4805</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>basileu.tavares@gmail.com</t>
+        </is>
+      </c>
+      <c r="I16" s="30" t="inlineStr">
+        <is>
+          <t>Basileu Pereira Tavares</t>
+        </is>
+      </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t>Luiza Bárbara Viana da Rocha (Sec. Finanças)</t>
         </is>
       </c>
       <c r="K16" s="28" t="inlineStr">
@@ -2230,34 +2309,34 @@
           <t>Centro-Direita</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F18" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G18" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H18" s="24" t="inlineStr">
-        <is>
-          <t>psdb.org.br</t>
-        </is>
-      </c>
-      <c r="I18" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J18" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Rua José Bello, 325 - Apto 702 - Aeroporto  CEP 36038-340</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98856-0047</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>(32) 98856-0047</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>aresiojunior@gmail.com</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>Arésio Ribeiro da Silva Júnior</t>
+        </is>
+      </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K18" s="28" t="inlineStr">
@@ -2293,34 +2372,34 @@
           <t>Direita</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
-        <is>
-          <t>Preencher via SGIP</t>
-        </is>
-      </c>
-      <c r="F19" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="G19" s="24" t="inlineStr">
-        <is>
-          <t>(32) Preencher</t>
-        </is>
-      </c>
-      <c r="H19" s="24" t="inlineStr">
-        <is>
-          <t>novo.org.br/diretorios</t>
-        </is>
-      </c>
-      <c r="I19" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
-        </is>
-      </c>
-      <c r="J19" s="24" t="inlineStr">
-        <is>
-          <t>Preencher</t>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Rua Ataliba de Barros, 182 - Sala 1109 - São Mateus  CEP 36025-275</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>(32) 98886-1838</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>(32) 98886-1838</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>juizdefora.mg@novo.org.br</t>
+        </is>
+      </c>
+      <c r="I19" s="30" t="inlineStr">
+        <is>
+          <t>Igor Burkowski</t>
+        </is>
+      </c>
+      <c r="J19" s="30" t="inlineStr">
+        <is>
+          <t>Contatar presidente</t>
         </is>
       </c>
       <c r="K19" s="25" t="inlineStr">
@@ -2526,19 +2605,102 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>LEGENDA PRIORIDADE:  ALTA = partido presidenciavel + 2+ vereadores  |  MEDIA = 1-2 vereadores  |  BAIXA = sem vereador ou partido menor</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>Como preencher: 1) Acesse sgip3.tse.jus.br  2) Selecione MG &gt; Juiz de Fora &gt; Partido  3) Copie endereco e dirigentes  4) Confirme por telefone com a sede</t>
-        </is>
-      </c>
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="50" t="inlineStr">
+        <is>
+          <t>PSOL</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Partido Socialismo e Liberdade</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Esquerda</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>Rua Dr. Hameleto Fellet, 101 - Apto 201 - Vale do Ipê  CEP 36036-130</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99175-5739</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>(32) 99175-5739</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>com.psoljf@gmail.com</t>
+        </is>
+      </c>
+      <c r="I23" s="30" t="inlineStr">
+        <is>
+          <t>Lorene Figueiredo de Oliveira</t>
+        </is>
+      </c>
+      <c r="J23" s="30" t="inlineStr">
+        <is>
+          <t>Felipe José Alves Santos (1º Secretário)</t>
+        </is>
+      </c>
+      <c r="K23" s="19" t="inlineStr">
+        <is>
+          <t>Sem vereador em JF 2025-28</t>
+        </is>
+      </c>
+      <c r="L23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="51" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="48" t="n"/>
+      <c r="C24" s="48" t="n"/>
+      <c r="D24" s="48" t="n"/>
+      <c r="E24" s="48" t="n"/>
+      <c r="F24" s="48" t="n"/>
+      <c r="G24" s="48" t="n"/>
+      <c r="H24" s="48" t="n"/>
+      <c r="I24" s="48" t="n"/>
+      <c r="J24" s="48" t="n"/>
+      <c r="K24" s="48" t="n"/>
+      <c r="L24" s="48" t="n"/>
+      <c r="M24" s="49" t="n"/>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="48" t="n"/>
+      <c r="C25" s="48" t="n"/>
+      <c r="D25" s="48" t="n"/>
+      <c r="E25" s="48" t="n"/>
+      <c r="F25" s="48" t="n"/>
+      <c r="G25" s="48" t="n"/>
+      <c r="H25" s="48" t="n"/>
+      <c r="I25" s="48" t="n"/>
+      <c r="J25" s="48" t="n"/>
+      <c r="K25" s="48" t="n"/>
+      <c r="L25" s="48" t="n"/>
+      <c r="M25" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2981,6 +3143,17 @@
           <t>STATUS:  Primeiro contato  |  Em negociacao  |  Reuniao agendada  |  Proposta enviada  |  Contrato fechado  |  Sem interesse  |  Follow-up pendente</t>
         </is>
       </c>
+      <c r="B29" s="48" t="n"/>
+      <c r="C29" s="48" t="n"/>
+      <c r="D29" s="48" t="n"/>
+      <c r="E29" s="48" t="n"/>
+      <c r="F29" s="48" t="n"/>
+      <c r="G29" s="48" t="n"/>
+      <c r="H29" s="48" t="n"/>
+      <c r="I29" s="48" t="n"/>
+      <c r="J29" s="48" t="n"/>
+      <c r="K29" s="48" t="n"/>
+      <c r="L29" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3029,6 +3202,7 @@
           <t>Total de Partidos Mapeados</t>
         </is>
       </c>
+      <c r="C4" s="49" t="n"/>
       <c r="D4" s="34" t="inlineStr">
         <is>
           <t>18</t>
@@ -3041,6 +3215,7 @@
           <t>Prioridade ALTA (3+ vereadores)</t>
         </is>
       </c>
+      <c r="C5" s="49" t="n"/>
       <c r="D5" s="36" t="inlineStr">
         <is>
           <t>3</t>
@@ -3053,6 +3228,7 @@
           <t>Prioridade MEDIA (1-2 vereadores)</t>
         </is>
       </c>
+      <c r="C6" s="49" t="n"/>
       <c r="D6" s="38" t="inlineStr">
         <is>
           <t>10</t>
@@ -3065,6 +3241,7 @@
           <t>Prioridade BAIXA (0 vereadores)</t>
         </is>
       </c>
+      <c r="C7" s="49" t="n"/>
       <c r="D7" s="40" t="inlineStr">
         <is>
           <t>5</t>
@@ -3077,6 +3254,7 @@
           <t>Contatos Realizados</t>
         </is>
       </c>
+      <c r="C8" s="49" t="n"/>
       <c r="D8" s="42" t="inlineStr">
         <is>
           <t>Preencher</t>
@@ -3089,6 +3267,7 @@
           <t>Reunioes Agendadas</t>
         </is>
       </c>
+      <c r="C9" s="49" t="n"/>
       <c r="D9" s="40" t="inlineStr">
         <is>
           <t>Preencher</t>
@@ -3101,6 +3280,7 @@
           <t>Propostas Enviadas</t>
         </is>
       </c>
+      <c r="C10" s="49" t="n"/>
       <c r="D10" s="38" t="inlineStr">
         <is>
           <t>Preencher</t>
@@ -3113,6 +3293,7 @@
           <t>Contratos Fechados</t>
         </is>
       </c>
+      <c r="C11" s="49" t="n"/>
       <c r="D11" s="40" t="inlineStr">
         <is>
           <t>Preencher</t>
@@ -3126,6 +3307,9 @@
           <t>CHECKLIST SEMANAL DE PROSPECCAO</t>
         </is>
       </c>
+      <c r="C14" s="48" t="n"/>
+      <c r="D14" s="48" t="n"/>
+      <c r="E14" s="49" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="44" t="inlineStr">
@@ -3133,6 +3317,9 @@
           <t>[ ] Verificar novas noticias sobre partidos em JF (Tribuna de Minas, Acessa.com)</t>
         </is>
       </c>
+      <c r="C15" s="48" t="n"/>
+      <c r="D15" s="48" t="n"/>
+      <c r="E15" s="49" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="45" t="inlineStr">
@@ -3140,6 +3327,9 @@
           <t>[ ] Atualizar CRM com contatos da semana (aba CRM Prospeccao)</t>
         </is>
       </c>
+      <c r="C16" s="48" t="n"/>
+      <c r="D16" s="48" t="n"/>
+      <c r="E16" s="49" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="44" t="inlineStr">
@@ -3147,6 +3337,9 @@
           <t>[ ] Enviar follow-up para contatos sem resposta ha mais de 7 dias</t>
         </is>
       </c>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="48" t="n"/>
+      <c r="E17" s="49" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="45" t="inlineStr">
@@ -3154,6 +3347,9 @@
           <t>[ ] Pesquisar no SGIP dados pendentes dos partidos (aba Partidos JF)</t>
         </is>
       </c>
+      <c r="C18" s="48" t="n"/>
+      <c r="D18" s="48" t="n"/>
+      <c r="E18" s="49" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="44" t="inlineStr">
@@ -3161,6 +3357,9 @@
           <t>[ ] Confirmar agenda de eventos politicos em JF na semana seguinte</t>
         </is>
       </c>
+      <c r="C19" s="48" t="n"/>
+      <c r="D19" s="48" t="n"/>
+      <c r="E19" s="49" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="B20" s="45" t="inlineStr">
@@ -3168,6 +3367,9 @@
           <t>[ ] Atualizar status dos 10 passos (aba Caminho Pratico)</t>
         </is>
       </c>
+      <c r="C20" s="48" t="n"/>
+      <c r="D20" s="48" t="n"/>
+      <c r="E20" s="49" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="44" t="inlineStr">
@@ -3175,6 +3377,9 @@
           <t>[ ] Revisar propostas enviadas e negociacoes abertas</t>
         </is>
       </c>
+      <c r="C21" s="48" t="n"/>
+      <c r="D21" s="48" t="n"/>
+      <c r="E21" s="49" t="n"/>
     </row>
     <row r="23" ht="10" customHeight="1"/>
     <row r="24" ht="28" customHeight="1">
@@ -3183,6 +3388,9 @@
           <t>DATAS CRITICAS 2026</t>
         </is>
       </c>
+      <c r="C24" s="48" t="n"/>
+      <c r="D24" s="48" t="n"/>
+      <c r="E24" s="49" t="n"/>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="B25" s="47" t="inlineStr">
@@ -3195,6 +3403,8 @@
           <t>AGORA - Equipes de campanha sendo formadas. Momento IDEAL para prospeccao.</t>
         </is>
       </c>
+      <c r="D25" s="48" t="n"/>
+      <c r="E25" s="49" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="B26" s="13" t="inlineStr">
@@ -3207,6 +3417,8 @@
           <t>Convencoes partidarias - candidaturas oficializadas. Ultima chance de entrada.</t>
         </is>
       </c>
+      <c r="D26" s="48" t="n"/>
+      <c r="E26" s="49" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="B27" s="47" t="inlineStr">
@@ -3219,6 +3431,8 @@
           <t>PRIMEIRO TURNO das eleicoes</t>
         </is>
       </c>
+      <c r="D27" s="48" t="n"/>
+      <c r="E27" s="49" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="B28" s="13" t="inlineStr">
@@ -3231,6 +3445,8 @@
           <t>SEGUNDO TURNO das eleicoes</t>
         </is>
       </c>
+      <c r="D28" s="48" t="n"/>
+      <c r="E28" s="49" t="n"/>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="B29" s="47" t="inlineStr">
@@ -3243,6 +3459,8 @@
           <t>Prestacao de contas no TSE - mapear quem foi contratado para 2030</t>
         </is>
       </c>
+      <c r="D29" s="48" t="n"/>
+      <c r="E29" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>